<commit_message>
Ajout de produits (2 nouveau(x)) dans CADENCIER.xlsx
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8711" uniqueCount="4415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8719" uniqueCount="4418">
   <si>
     <t>Code barre</t>
   </si>
@@ -13256,6 +13256,15 @@
   </si>
   <si>
     <t>SORBET MANGUE PASSION 125ML</t>
+  </si>
+  <si>
+    <t>9661234100259</t>
+  </si>
+  <si>
+    <t>PAPIER HYGIENIQUE DOUCY ECO P12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOCIETE DE PRODUCTION D'ARTICLES </t>
   </si>
 </sst>
 </file>
@@ -13632,7 +13641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2177"/>
+  <dimension ref="A1:E2179"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -50644,6 +50653,40 @@
         <v>3362</v>
       </c>
     </row>
+    <row r="2178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2178" t="s">
+        <v>4415</v>
+      </c>
+      <c r="B2178">
+        <v>50042318</v>
+      </c>
+      <c r="C2178" t="s">
+        <v>4416</v>
+      </c>
+      <c r="D2178" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2178" t="s">
+        <v>4417</v>
+      </c>
+    </row>
+    <row r="2179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2179" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2179">
+        <v>50042319</v>
+      </c>
+      <c r="C2179" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2179" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2179" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Mise à jour CADENCIER.xlsx
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8719" uniqueCount="4418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8711" uniqueCount="4415">
   <si>
     <t>Code barre</t>
   </si>
@@ -13256,15 +13256,6 @@
   </si>
   <si>
     <t>SORBET MANGUE PASSION 125ML</t>
-  </si>
-  <si>
-    <t>9661234100259</t>
-  </si>
-  <si>
-    <t>PAPIER HYGIENIQUE DOUCY ECO P12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOCIETE DE PRODUCTION D'ARTICLES </t>
   </si>
 </sst>
 </file>
@@ -13641,7 +13632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2179"/>
+  <dimension ref="A1:E2177"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -50653,40 +50644,6 @@
         <v>3362</v>
       </c>
     </row>
-    <row r="2178" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2178" t="s">
-        <v>4415</v>
-      </c>
-      <c r="B2178">
-        <v>50042318</v>
-      </c>
-      <c r="C2178" t="s">
-        <v>4416</v>
-      </c>
-      <c r="D2178" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2178" t="s">
-        <v>4417</v>
-      </c>
-    </row>
-    <row r="2179" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2179" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2179">
-        <v>50042319</v>
-      </c>
-      <c r="C2179" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2179" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2179" t="s">
-        <v>9</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout de produits dans CADENCIER.xlsx – 2 nouveau(x)
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8711" uniqueCount="4415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8719" uniqueCount="4418">
   <si>
     <t>Code barre</t>
   </si>
@@ -13256,6 +13256,15 @@
   </si>
   <si>
     <t>SORBET MANGUE PASSION 125ML</t>
+  </si>
+  <si>
+    <t>9661234100259</t>
+  </si>
+  <si>
+    <t>PAPIER HYGIENIQUE DOUCY ECO P12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOCIETE DE PRODUCTION D'ARTICLES </t>
   </si>
 </sst>
 </file>
@@ -13632,7 +13641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2177"/>
+  <dimension ref="A1:E2179"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -50644,6 +50653,40 @@
         <v>3362</v>
       </c>
     </row>
+    <row r="2178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2178" t="s">
+        <v>4415</v>
+      </c>
+      <c r="B2178">
+        <v>50042318</v>
+      </c>
+      <c r="C2178" t="s">
+        <v>4416</v>
+      </c>
+      <c r="D2178" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2178" t="s">
+        <v>4417</v>
+      </c>
+    </row>
+    <row r="2179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2179" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2179">
+        <v>50042319</v>
+      </c>
+      <c r="C2179" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2179" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2179" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout CADENCIER.xlsx – 2 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8711" uniqueCount="4415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8719" uniqueCount="4418">
   <si>
     <t>Code barre</t>
   </si>
@@ -13256,6 +13256,15 @@
   </si>
   <si>
     <t>SORBET MANGUE PASSION 125ML</t>
+  </si>
+  <si>
+    <t>9661234100259</t>
+  </si>
+  <si>
+    <t>PAPIER HYGIENIQUE DOUCY ECO P12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOCIETE DE PRODUCTION D'ARTICLES </t>
   </si>
 </sst>
 </file>
@@ -13632,7 +13641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2177"/>
+  <dimension ref="A1:E2179"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -50644,6 +50653,40 @@
         <v>3362</v>
       </c>
     </row>
+    <row r="2178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2178" t="s">
+        <v>4415</v>
+      </c>
+      <c r="B2178">
+        <v>50042318</v>
+      </c>
+      <c r="C2178" t="s">
+        <v>4416</v>
+      </c>
+      <c r="D2178" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2178" t="s">
+        <v>4417</v>
+      </c>
+    </row>
+    <row r="2179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2179" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2179">
+        <v>50042319</v>
+      </c>
+      <c r="C2179" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2179" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2179" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout CADENCIER.xlsx – 1 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8719" uniqueCount="4418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8721" uniqueCount="4420">
   <si>
     <t>Code barre</t>
   </si>
@@ -13265,6 +13265,12 @@
   </si>
   <si>
     <t xml:space="preserve">SOCIETE DE PRODUCTION D'ARTICLES </t>
+  </si>
+  <si>
+    <t>io</t>
+  </si>
+  <si>
+    <t>Andrana</t>
   </si>
 </sst>
 </file>
@@ -13641,7 +13647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2179"/>
+  <dimension ref="A1:E2180"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -50687,6 +50693,23 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2180">
+        <v>5321</v>
+      </c>
+      <c r="B2180">
+        <v>12345</v>
+      </c>
+      <c r="C2180" t="s">
+        <v>4418</v>
+      </c>
+      <c r="D2180">
+        <v>30</v>
+      </c>
+      <c r="E2180" t="s">
+        <v>4419</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout CADENCIER.xlsx – 40 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8721" uniqueCount="4420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8801" uniqueCount="4462">
   <si>
     <t>Code barre</t>
   </si>
@@ -13271,6 +13271,132 @@
   </si>
   <si>
     <t>Andrana</t>
+  </si>
+  <si>
+    <t>PUREE DE PIMENT ROUGE 100G</t>
+  </si>
+  <si>
+    <t>CODAL</t>
+  </si>
+  <si>
+    <t>PUREE DE PIMENT VERT 100G</t>
+  </si>
+  <si>
+    <t>PUREE DE PIMENT VERT 200G</t>
+  </si>
+  <si>
+    <t>PUREE DE PIMENT ROUGE 200G</t>
+  </si>
+  <si>
+    <t>PUREE DE PIMENT AU POIVRE SAUVAGE 100G</t>
+  </si>
+  <si>
+    <t>PUREE DE PIMENT AU COMBAVA 100G</t>
+  </si>
+  <si>
+    <t>RAVITOTO 420G</t>
+  </si>
+  <si>
+    <t>RAVITOTO COCO 420G</t>
+  </si>
+  <si>
+    <t>ACHARDS DE LEGUMES 130G</t>
+  </si>
+  <si>
+    <t>ACHARDS DE LEGUMES 400G</t>
+  </si>
+  <si>
+    <t>MOUTARDES  AROMATISEES À L'AIL 200G</t>
+  </si>
+  <si>
+    <t>MOUTARDES  AROMATISEES AU COMBAVA 200G</t>
+  </si>
+  <si>
+    <t>CITRONNELLE  FEUILLES BIO 50G</t>
+  </si>
+  <si>
+    <t>HIBISCUS FLEURS SECHEES BIO 50G</t>
+  </si>
+  <si>
+    <t>HIBISCUS FLEURS SECHEES BIO 100G</t>
+  </si>
+  <si>
+    <t>PICOLO CONFITURE  FRAISE 150G</t>
+  </si>
+  <si>
+    <t>PICOLO CONFITURE  TUTTI FRUITI 150G</t>
+  </si>
+  <si>
+    <t>PICOLO CONFITURE  PRUNE 150G</t>
+  </si>
+  <si>
+    <t>PICOLO CONFITURE  GOYAVE 150G</t>
+  </si>
+  <si>
+    <t>PICOLO COMPTOTE NATURE 150G</t>
+  </si>
+  <si>
+    <t>PICOLO COMPOTE POMMES BANANES 150G</t>
+  </si>
+  <si>
+    <t>PICOLO COMPOTE  POMMES FRAISES 150G</t>
+  </si>
+  <si>
+    <t>PICOLO COMPOTE POMMES EXOTIQUE 150G</t>
+  </si>
+  <si>
+    <t>CONFITURE  FRAISE 220G</t>
+  </si>
+  <si>
+    <t>CONFITURE  POKPOK 220G</t>
+  </si>
+  <si>
+    <t>CONFITURE  MURES 220G</t>
+  </si>
+  <si>
+    <t>CONFITURE  ORANGE 220G</t>
+  </si>
+  <si>
+    <t>SOAÏRA CHOCOLAT AU LAIT 45% AVEC PRALINE CACAHUETE 100G</t>
+  </si>
+  <si>
+    <t>SOAVA CHOCOLAT AU LAIT 33% AVEC PRALINE CAJOU 100G</t>
+  </si>
+  <si>
+    <t>MANIVA CHOCOLAT AU LAIT 33% GANACHE VANILLE 100G</t>
+  </si>
+  <si>
+    <t>VOANIA CHOCOLAT AU LAIT 45% AVE ÉCLATS DE NOIX DE COCO 75G</t>
+  </si>
+  <si>
+    <t>NOSIKO CHOCOLAT AU LAIT 33% 75G</t>
+  </si>
+  <si>
+    <t>CHAMPIGNON PARFUME 250GR SHIITAKE</t>
+  </si>
+  <si>
+    <t>YOPLAIT YAOURT A BOIRE VANILLE EN SACHET 70G</t>
+  </si>
+  <si>
+    <t>PANAGORA</t>
+  </si>
+  <si>
+    <t>YOPLAIT YAOURT A BOIRE FRASE EN SACHET 70G</t>
+  </si>
+  <si>
+    <t>BIBERON ZAZA COMPLET VERRE 120ML</t>
+  </si>
+  <si>
+    <t>BIBERON ZAZA COMPLET VERRE 240ML</t>
+  </si>
+  <si>
+    <t>TETINE ZAZA SILICONE ANTI-COLIQUE L (+6 MOIS)</t>
+  </si>
+  <si>
+    <t>TETINE ZAZA SILICONE ANTI-COLIQUE M (3-6 MOIS)</t>
+  </si>
+  <si>
+    <t>TETINE ZAZA SILICONE ANTI-COLIQUE S (0-3 MOIS)</t>
   </si>
 </sst>
 </file>
@@ -13647,7 +13773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2180"/>
+  <dimension ref="A1:E2220"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -50710,6 +50836,686 @@
         <v>4419</v>
       </c>
     </row>
+    <row r="2181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2181">
+        <v>3760153582415</v>
+      </c>
+      <c r="B2181">
+        <v>50043101</v>
+      </c>
+      <c r="C2181" t="s">
+        <v>4420</v>
+      </c>
+      <c r="D2181">
+        <v>24</v>
+      </c>
+      <c r="E2181" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2182">
+        <v>3760153582422</v>
+      </c>
+      <c r="B2182">
+        <v>50043102</v>
+      </c>
+      <c r="C2182" t="s">
+        <v>4422</v>
+      </c>
+      <c r="D2182">
+        <v>24</v>
+      </c>
+      <c r="E2182" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2183">
+        <v>3760153584372</v>
+      </c>
+      <c r="B2183">
+        <v>71093221</v>
+      </c>
+      <c r="C2183" t="s">
+        <v>4423</v>
+      </c>
+      <c r="D2183">
+        <v>12</v>
+      </c>
+      <c r="E2183" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2184">
+        <v>3760153584389</v>
+      </c>
+      <c r="B2184">
+        <v>71093222</v>
+      </c>
+      <c r="C2184" t="s">
+        <v>4424</v>
+      </c>
+      <c r="D2184">
+        <v>12</v>
+      </c>
+      <c r="E2184" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2185">
+        <v>3076017392022</v>
+      </c>
+      <c r="B2185">
+        <v>71093223</v>
+      </c>
+      <c r="C2185" t="s">
+        <v>4425</v>
+      </c>
+      <c r="D2185">
+        <v>24</v>
+      </c>
+      <c r="E2185" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2186">
+        <v>3760153599765</v>
+      </c>
+      <c r="B2186">
+        <v>71093224</v>
+      </c>
+      <c r="C2186" t="s">
+        <v>4426</v>
+      </c>
+      <c r="D2186">
+        <v>24</v>
+      </c>
+      <c r="E2186" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2187">
+        <v>3760153581791</v>
+      </c>
+      <c r="B2187">
+        <v>71093225</v>
+      </c>
+      <c r="C2187" t="s">
+        <v>4427</v>
+      </c>
+      <c r="D2187">
+        <v>12</v>
+      </c>
+      <c r="E2187" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2188">
+        <v>3760153599925</v>
+      </c>
+      <c r="B2188">
+        <v>71093226</v>
+      </c>
+      <c r="C2188" t="s">
+        <v>4428</v>
+      </c>
+      <c r="D2188">
+        <v>12</v>
+      </c>
+      <c r="E2188" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2189">
+        <v>3760153580992</v>
+      </c>
+      <c r="B2189">
+        <v>71093227</v>
+      </c>
+      <c r="C2189" t="s">
+        <v>4429</v>
+      </c>
+      <c r="D2189">
+        <v>24</v>
+      </c>
+      <c r="E2189" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2190">
+        <v>3760153583443</v>
+      </c>
+      <c r="B2190">
+        <v>71093228</v>
+      </c>
+      <c r="C2190" t="s">
+        <v>4430</v>
+      </c>
+      <c r="D2190">
+        <v>24</v>
+      </c>
+      <c r="E2190" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2191">
+        <v>3760153581487</v>
+      </c>
+      <c r="B2191">
+        <v>71093229</v>
+      </c>
+      <c r="C2191" t="s">
+        <v>4431</v>
+      </c>
+      <c r="D2191">
+        <v>12</v>
+      </c>
+      <c r="E2191" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2192">
+        <v>3760153581494</v>
+      </c>
+      <c r="B2192">
+        <v>71093230</v>
+      </c>
+      <c r="C2192" t="s">
+        <v>4432</v>
+      </c>
+      <c r="D2192">
+        <v>12</v>
+      </c>
+      <c r="E2192" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2193">
+        <v>3760153590109</v>
+      </c>
+      <c r="B2193">
+        <v>71093231</v>
+      </c>
+      <c r="C2193" t="s">
+        <v>4433</v>
+      </c>
+      <c r="D2193">
+        <v>10</v>
+      </c>
+      <c r="E2193" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2194">
+        <v>3760153599048</v>
+      </c>
+      <c r="B2194">
+        <v>71093232</v>
+      </c>
+      <c r="C2194" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D2194">
+        <v>12</v>
+      </c>
+      <c r="E2194" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2195">
+        <v>3760153599031</v>
+      </c>
+      <c r="B2195">
+        <v>71093233</v>
+      </c>
+      <c r="C2195" t="s">
+        <v>4435</v>
+      </c>
+      <c r="D2195">
+        <v>12</v>
+      </c>
+      <c r="E2195" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2196">
+        <v>3760153599086</v>
+      </c>
+      <c r="B2196">
+        <v>71093234</v>
+      </c>
+      <c r="C2196" t="s">
+        <v>4436</v>
+      </c>
+      <c r="D2196">
+        <v>24</v>
+      </c>
+      <c r="E2196" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2197">
+        <v>3760153599079</v>
+      </c>
+      <c r="B2197">
+        <v>71093235</v>
+      </c>
+      <c r="C2197" t="s">
+        <v>4437</v>
+      </c>
+      <c r="D2197">
+        <v>24</v>
+      </c>
+      <c r="E2197" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2198">
+        <v>3760153599093</v>
+      </c>
+      <c r="B2198">
+        <v>71093236</v>
+      </c>
+      <c r="C2198" t="s">
+        <v>4438</v>
+      </c>
+      <c r="D2198">
+        <v>24</v>
+      </c>
+      <c r="E2198" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2199">
+        <v>3760153599062</v>
+      </c>
+      <c r="B2199">
+        <v>71093237</v>
+      </c>
+      <c r="C2199" t="s">
+        <v>4439</v>
+      </c>
+      <c r="D2199">
+        <v>24</v>
+      </c>
+      <c r="E2199" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2200">
+        <v>3760153599246</v>
+      </c>
+      <c r="B2200">
+        <v>71093238</v>
+      </c>
+      <c r="C2200" t="s">
+        <v>4440</v>
+      </c>
+      <c r="D2200">
+        <v>24</v>
+      </c>
+      <c r="E2200" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2201">
+        <v>3760153599253</v>
+      </c>
+      <c r="B2201">
+        <v>71093239</v>
+      </c>
+      <c r="C2201" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D2201">
+        <v>24</v>
+      </c>
+      <c r="E2201" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2202">
+        <v>3760153599260</v>
+      </c>
+      <c r="B2202">
+        <v>71093240</v>
+      </c>
+      <c r="C2202" t="s">
+        <v>4442</v>
+      </c>
+      <c r="D2202">
+        <v>24</v>
+      </c>
+      <c r="E2202" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2203">
+        <v>3760153599277</v>
+      </c>
+      <c r="B2203">
+        <v>71093241</v>
+      </c>
+      <c r="C2203" t="s">
+        <v>4443</v>
+      </c>
+      <c r="D2203">
+        <v>24</v>
+      </c>
+      <c r="E2203" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2204">
+        <v>3076017391025</v>
+      </c>
+      <c r="B2204">
+        <v>71093242</v>
+      </c>
+      <c r="C2204" t="s">
+        <v>4444</v>
+      </c>
+      <c r="D2204">
+        <v>12</v>
+      </c>
+      <c r="E2204" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2205">
+        <v>3073017391100</v>
+      </c>
+      <c r="B2205">
+        <v>71093243</v>
+      </c>
+      <c r="C2205" t="s">
+        <v>4445</v>
+      </c>
+      <c r="D2205">
+        <v>12</v>
+      </c>
+      <c r="E2205" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2206">
+        <v>3076017391049</v>
+      </c>
+      <c r="B2206">
+        <v>71093244</v>
+      </c>
+      <c r="C2206" t="s">
+        <v>4446</v>
+      </c>
+      <c r="D2206">
+        <v>12</v>
+      </c>
+      <c r="E2206" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2207">
+        <v>3076017391070</v>
+      </c>
+      <c r="B2207">
+        <v>71093245</v>
+      </c>
+      <c r="C2207" t="s">
+        <v>4447</v>
+      </c>
+      <c r="D2207">
+        <v>12</v>
+      </c>
+      <c r="E2207" t="s">
+        <v>4421</v>
+      </c>
+    </row>
+    <row r="2208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2208">
+        <v>619091605140</v>
+      </c>
+      <c r="B2208">
+        <v>71093246</v>
+      </c>
+      <c r="C2208" t="s">
+        <v>4448</v>
+      </c>
+      <c r="D2208">
+        <v>10</v>
+      </c>
+      <c r="E2208" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="2209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2209">
+        <v>619091605157</v>
+      </c>
+      <c r="B2209">
+        <v>71093247</v>
+      </c>
+      <c r="C2209" t="s">
+        <v>4449</v>
+      </c>
+      <c r="D2209">
+        <v>10</v>
+      </c>
+      <c r="E2209" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="2210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2210">
+        <v>619091605188</v>
+      </c>
+      <c r="B2210">
+        <v>71093248</v>
+      </c>
+      <c r="C2210" t="s">
+        <v>4450</v>
+      </c>
+      <c r="D2210">
+        <v>10</v>
+      </c>
+      <c r="E2210" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="2211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2211">
+        <v>619091605126</v>
+      </c>
+      <c r="B2211">
+        <v>71093249</v>
+      </c>
+      <c r="C2211" t="s">
+        <v>4451</v>
+      </c>
+      <c r="D2211">
+        <v>10</v>
+      </c>
+      <c r="E2211" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="2212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2212">
+        <v>619091605133</v>
+      </c>
+      <c r="B2212">
+        <v>71093250</v>
+      </c>
+      <c r="C2212" t="s">
+        <v>4452</v>
+      </c>
+      <c r="D2212">
+        <v>10</v>
+      </c>
+      <c r="E2212" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="2213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2213">
+        <v>6091302492222</v>
+      </c>
+      <c r="B2213">
+        <v>71093251</v>
+      </c>
+      <c r="C2213" t="s">
+        <v>4453</v>
+      </c>
+      <c r="D2213">
+        <v>12</v>
+      </c>
+      <c r="E2213" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2214">
+        <v>6091002019156</v>
+      </c>
+      <c r="B2214">
+        <v>75093252</v>
+      </c>
+      <c r="C2214" t="s">
+        <v>4454</v>
+      </c>
+      <c r="D2214">
+        <v>10</v>
+      </c>
+      <c r="E2214" t="s">
+        <v>4455</v>
+      </c>
+    </row>
+    <row r="2215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2215">
+        <v>6091002019163</v>
+      </c>
+      <c r="B2215">
+        <v>75093253</v>
+      </c>
+      <c r="C2215" t="s">
+        <v>4456</v>
+      </c>
+      <c r="D2215">
+        <v>10</v>
+      </c>
+      <c r="E2215" t="s">
+        <v>4455</v>
+      </c>
+    </row>
+    <row r="2216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2216">
+        <v>6900004304170</v>
+      </c>
+      <c r="B2216">
+        <v>74093254</v>
+      </c>
+      <c r="C2216" t="s">
+        <v>4457</v>
+      </c>
+      <c r="D2216">
+        <v>1</v>
+      </c>
+      <c r="E2216" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2217">
+        <v>6900004018954</v>
+      </c>
+      <c r="B2217">
+        <v>74093255</v>
+      </c>
+      <c r="C2217" t="s">
+        <v>4458</v>
+      </c>
+      <c r="D2217">
+        <v>1</v>
+      </c>
+      <c r="E2217" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2218">
+        <v>6900004091094</v>
+      </c>
+      <c r="B2218">
+        <v>74093256</v>
+      </c>
+      <c r="C2218" t="s">
+        <v>4459</v>
+      </c>
+      <c r="D2218">
+        <v>1</v>
+      </c>
+      <c r="E2218" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2219">
+        <v>6900004191817</v>
+      </c>
+      <c r="B2219">
+        <v>74093257</v>
+      </c>
+      <c r="C2219" t="s">
+        <v>4460</v>
+      </c>
+      <c r="D2219">
+        <v>1</v>
+      </c>
+      <c r="E2219" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2220">
+        <v>6900004193026</v>
+      </c>
+      <c r="B2220">
+        <v>74093258</v>
+      </c>
+      <c r="C2220" t="s">
+        <v>4461</v>
+      </c>
+      <c r="D2220">
+        <v>1</v>
+      </c>
+      <c r="E2220" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout CADENCIER.xlsx – 38 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8801" uniqueCount="4462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8877" uniqueCount="4503">
   <si>
     <t>Code barre</t>
   </si>
@@ -13397,6 +13397,129 @@
   </si>
   <si>
     <t>TETINE ZAZA SILICONE ANTI-COLIQUE S (0-3 MOIS)</t>
+  </si>
+  <si>
+    <t>DIADERMINE SAVON DERMATOLOGIE 100G</t>
+  </si>
+  <si>
+    <t>DIADERMINE SAVON SURGRAS 100G</t>
+  </si>
+  <si>
+    <t>DIADERMINE PH 5 HYDRATANT PROTECTEUR DAY CREAM 50 ML</t>
+  </si>
+  <si>
+    <t>DIADERMINE PH 7 HYDRATANT MATIFIANT DAY CREAM 50 ML</t>
+  </si>
+  <si>
+    <t>MONT SAINT MICHEL BAR SOAP AMBREE 125G</t>
+  </si>
+  <si>
+    <t>MONT SAINT MICHEL BAR SOAP FRAICHEUR 125G</t>
+  </si>
+  <si>
+    <t>DENIVIT BLANCHEUR ET LUMIERE 50ML</t>
+  </si>
+  <si>
+    <t>DENIVIT BLANCHEUR SUBLIME 50ML</t>
+  </si>
+  <si>
+    <t>VADEMECUM FLUOR PLANTES 75ML</t>
+  </si>
+  <si>
+    <t>VADEMECUM PURETE ECALYPTUS 75ML</t>
+  </si>
+  <si>
+    <t>VADEMECUM BLANCHEUR ET PLANTES 75ML</t>
+  </si>
+  <si>
+    <t>ROYAL LEXI PEARL POWDER &amp; MILK 175G</t>
+  </si>
+  <si>
+    <t>ROYAL LEXI CREAM MILK 175G</t>
+  </si>
+  <si>
+    <t>ROYAL LEXI ROSE MILK 175G</t>
+  </si>
+  <si>
+    <t>ROYAL LEXI WHITE DIAMOND 175G</t>
+  </si>
+  <si>
+    <t>ROYAL LEXI FRESH GREEN 175G</t>
+  </si>
+  <si>
+    <t>ROYAL LEXI AQUA FRESH 175G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROYAL LEXI ROMANTIC 175G </t>
+  </si>
+  <si>
+    <t>AYAM TERIYAKI SAUCE 210ML</t>
+  </si>
+  <si>
+    <t>SICE</t>
+  </si>
+  <si>
+    <t>AYAM SWEET SOUR SAUCE 210ML</t>
+  </si>
+  <si>
+    <t>AYAM YAKITORI SAUCE 210ML</t>
+  </si>
+  <si>
+    <t>AYAM PONZU SAUCE 210ML</t>
+  </si>
+  <si>
+    <t>AYAM CARAMELIZED SOYA SUCE 210ML</t>
+  </si>
+  <si>
+    <t>AYAM GREEN CURRY PASTE 100G</t>
+  </si>
+  <si>
+    <t>AYAM RED CURRY PASTE 100G</t>
+  </si>
+  <si>
+    <t>BISCUIT BAKERY BUTTER 66G</t>
+  </si>
+  <si>
+    <t>BRITA</t>
+  </si>
+  <si>
+    <t>BISCUITS COCONUT 66G</t>
+  </si>
+  <si>
+    <t>BISCUITS LU GALA EGG 100GR</t>
+  </si>
+  <si>
+    <t>BISCUITS NANKHATAI BAKERI 84G</t>
+  </si>
+  <si>
+    <t>TOPPER CUSTARD 125G</t>
+  </si>
+  <si>
+    <t>AZIMA</t>
+  </si>
+  <si>
+    <t>TOPPER CHOCOLATE 125G</t>
+  </si>
+  <si>
+    <t>TOPPER VANILLA 125G</t>
+  </si>
+  <si>
+    <t>TOPPER RASPBERRY 125G</t>
+  </si>
+  <si>
+    <t>EET SUM MOR CHOCOLATE CHIPS 200G</t>
+  </si>
+  <si>
+    <t>EET SUM MOR EXP 200G</t>
+  </si>
+  <si>
+    <t>EET SUM MOR 80G</t>
+  </si>
+  <si>
+    <t>TEA LATTE  GREEN MATCHA 240G</t>
+  </si>
+  <si>
+    <t>FARINE MULTIUSAGE FIONA 1KG</t>
   </si>
 </sst>
 </file>
@@ -13773,7 +13896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2220"/>
+  <dimension ref="A1:E2258"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -51516,6 +51639,652 @@
         <v>87</v>
       </c>
     </row>
+    <row r="2221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2221">
+        <v>3178040584679</v>
+      </c>
+      <c r="B2221">
+        <v>50042450</v>
+      </c>
+      <c r="C2221" t="s">
+        <v>4462</v>
+      </c>
+      <c r="D2221">
+        <v>13500</v>
+      </c>
+      <c r="E2221" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2222">
+        <v>3178040585515</v>
+      </c>
+      <c r="B2222">
+        <v>50042451</v>
+      </c>
+      <c r="C2222" t="s">
+        <v>4463</v>
+      </c>
+      <c r="D2222">
+        <v>13500</v>
+      </c>
+      <c r="E2222" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2223">
+        <v>3178044048528</v>
+      </c>
+      <c r="B2223">
+        <v>50042653</v>
+      </c>
+      <c r="C2223" t="s">
+        <v>4464</v>
+      </c>
+      <c r="D2223">
+        <v>22500</v>
+      </c>
+      <c r="E2223" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2224">
+        <v>3178044048535</v>
+      </c>
+      <c r="B2224">
+        <v>50042654</v>
+      </c>
+      <c r="C2224" t="s">
+        <v>4465</v>
+      </c>
+      <c r="D2224">
+        <v>22500</v>
+      </c>
+      <c r="E2224" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2225">
+        <v>3178040666283</v>
+      </c>
+      <c r="B2225">
+        <v>73093384</v>
+      </c>
+      <c r="C2225" t="s">
+        <v>4466</v>
+      </c>
+      <c r="D2225">
+        <v>10900</v>
+      </c>
+      <c r="E2225" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2226">
+        <v>3178040666290</v>
+      </c>
+      <c r="B2226">
+        <v>73093385</v>
+      </c>
+      <c r="C2226" t="s">
+        <v>4467</v>
+      </c>
+      <c r="D2226">
+        <v>10900</v>
+      </c>
+      <c r="E2226" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2227">
+        <v>4068881000140</v>
+      </c>
+      <c r="B2227">
+        <v>50048662</v>
+      </c>
+      <c r="C2227" t="s">
+        <v>4468</v>
+      </c>
+      <c r="D2227">
+        <v>12500</v>
+      </c>
+      <c r="E2227" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2228">
+        <v>4068881000201</v>
+      </c>
+      <c r="B2228">
+        <v>50048663</v>
+      </c>
+      <c r="C2228" t="s">
+        <v>4469</v>
+      </c>
+      <c r="D2228">
+        <v>12500</v>
+      </c>
+      <c r="E2228" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2229" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2229">
+        <v>4068883000216</v>
+      </c>
+      <c r="B2229">
+        <v>50042544</v>
+      </c>
+      <c r="C2229" t="s">
+        <v>4470</v>
+      </c>
+      <c r="D2229">
+        <v>11500</v>
+      </c>
+      <c r="E2229" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2230">
+        <v>4068883000780</v>
+      </c>
+      <c r="B2230">
+        <v>50042546</v>
+      </c>
+      <c r="C2230" t="s">
+        <v>4471</v>
+      </c>
+      <c r="D2230">
+        <v>11500</v>
+      </c>
+      <c r="E2230" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2231">
+        <v>4068883000230</v>
+      </c>
+      <c r="B2231">
+        <v>73093386</v>
+      </c>
+      <c r="C2231" t="s">
+        <v>4472</v>
+      </c>
+      <c r="D2231">
+        <v>11500</v>
+      </c>
+      <c r="E2231" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2232">
+        <v>8997220606667</v>
+      </c>
+      <c r="B2232">
+        <v>73093387</v>
+      </c>
+      <c r="C2232" t="s">
+        <v>4473</v>
+      </c>
+      <c r="D2232">
+        <v>3990</v>
+      </c>
+      <c r="E2232" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2233">
+        <v>8997220606698</v>
+      </c>
+      <c r="B2233">
+        <v>73093388</v>
+      </c>
+      <c r="C2233" t="s">
+        <v>4474</v>
+      </c>
+      <c r="D2233">
+        <v>3990</v>
+      </c>
+      <c r="E2233" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2234">
+        <v>8997220606650</v>
+      </c>
+      <c r="B2234">
+        <v>73093389</v>
+      </c>
+      <c r="C2234" t="s">
+        <v>4475</v>
+      </c>
+      <c r="D2234">
+        <v>3990</v>
+      </c>
+      <c r="E2234" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2235">
+        <v>8997220606704</v>
+      </c>
+      <c r="B2235">
+        <v>73093390</v>
+      </c>
+      <c r="C2235" t="s">
+        <v>4476</v>
+      </c>
+      <c r="D2235">
+        <v>3990</v>
+      </c>
+      <c r="E2235" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2236" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2236">
+        <v>8997220606674</v>
+      </c>
+      <c r="B2236">
+        <v>73093391</v>
+      </c>
+      <c r="C2236" t="s">
+        <v>4477</v>
+      </c>
+      <c r="D2236">
+        <v>3990</v>
+      </c>
+      <c r="E2236" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2237" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2237">
+        <v>8997220606681</v>
+      </c>
+      <c r="B2237">
+        <v>73093392</v>
+      </c>
+      <c r="C2237" t="s">
+        <v>4478</v>
+      </c>
+      <c r="D2237">
+        <v>3990</v>
+      </c>
+      <c r="E2237" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2238" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2238">
+        <v>8997220609965</v>
+      </c>
+      <c r="B2238">
+        <v>73093393</v>
+      </c>
+      <c r="C2238" t="s">
+        <v>4479</v>
+      </c>
+      <c r="D2238">
+        <v>3990</v>
+      </c>
+      <c r="E2238" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2239" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2239">
+        <v>9556041611152</v>
+      </c>
+      <c r="B2239">
+        <v>71093394</v>
+      </c>
+      <c r="C2239" t="s">
+        <v>4480</v>
+      </c>
+      <c r="D2239">
+        <v>12300</v>
+      </c>
+      <c r="E2239" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2240">
+        <v>9556041611121</v>
+      </c>
+      <c r="B2240">
+        <v>71093395</v>
+      </c>
+      <c r="C2240" t="s">
+        <v>4482</v>
+      </c>
+      <c r="D2240">
+        <v>13000</v>
+      </c>
+      <c r="E2240" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2241">
+        <v>9556041132411</v>
+      </c>
+      <c r="B2241">
+        <v>71093396</v>
+      </c>
+      <c r="C2241" t="s">
+        <v>4483</v>
+      </c>
+      <c r="D2241">
+        <v>12300</v>
+      </c>
+      <c r="E2241" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2242" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2242">
+        <v>9556041132664</v>
+      </c>
+      <c r="B2242">
+        <v>71093397</v>
+      </c>
+      <c r="C2242" t="s">
+        <v>4484</v>
+      </c>
+      <c r="D2242">
+        <v>10500</v>
+      </c>
+      <c r="E2242" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2243">
+        <v>9556041613620</v>
+      </c>
+      <c r="B2243">
+        <v>71093398</v>
+      </c>
+      <c r="C2243" t="s">
+        <v>4485</v>
+      </c>
+      <c r="D2243">
+        <v>11500</v>
+      </c>
+      <c r="E2243" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2244">
+        <v>9556041780612</v>
+      </c>
+      <c r="B2244">
+        <v>71093399</v>
+      </c>
+      <c r="C2244" t="s">
+        <v>4486</v>
+      </c>
+      <c r="D2244">
+        <v>8500</v>
+      </c>
+      <c r="E2244" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2245">
+        <v>9556041780629</v>
+      </c>
+      <c r="B2245">
+        <v>71093400</v>
+      </c>
+      <c r="C2245" t="s">
+        <v>4487</v>
+      </c>
+      <c r="D2245">
+        <v>8500</v>
+      </c>
+      <c r="E2245" t="s">
+        <v>4481</v>
+      </c>
+    </row>
+    <row r="2246" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2246">
+        <v>8961003011740</v>
+      </c>
+      <c r="B2246">
+        <v>71093401</v>
+      </c>
+      <c r="C2246" t="s">
+        <v>4488</v>
+      </c>
+      <c r="D2246">
+        <v>4000</v>
+      </c>
+      <c r="E2246" t="s">
+        <v>4489</v>
+      </c>
+    </row>
+    <row r="2247" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2247">
+        <v>8961003011733</v>
+      </c>
+      <c r="B2247">
+        <v>71093402</v>
+      </c>
+      <c r="C2247" t="s">
+        <v>4490</v>
+      </c>
+      <c r="D2247">
+        <v>4000</v>
+      </c>
+      <c r="E2247" t="s">
+        <v>4489</v>
+      </c>
+    </row>
+    <row r="2248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2248">
+        <v>8961003010521</v>
+      </c>
+      <c r="B2248">
+        <v>71093403</v>
+      </c>
+      <c r="C2248" t="s">
+        <v>4491</v>
+      </c>
+      <c r="D2248">
+        <v>4000</v>
+      </c>
+      <c r="E2248" t="s">
+        <v>4489</v>
+      </c>
+    </row>
+    <row r="2249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2249">
+        <v>8961003011771</v>
+      </c>
+      <c r="B2249">
+        <v>71093404</v>
+      </c>
+      <c r="C2249" t="s">
+        <v>4492</v>
+      </c>
+      <c r="D2249">
+        <v>4000</v>
+      </c>
+      <c r="E2249" t="s">
+        <v>4489</v>
+      </c>
+    </row>
+    <row r="2250" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2250">
+        <v>6001056412940</v>
+      </c>
+      <c r="B2250">
+        <v>71093405</v>
+      </c>
+      <c r="C2250" t="s">
+        <v>4493</v>
+      </c>
+      <c r="D2250">
+        <v>4500</v>
+      </c>
+      <c r="E2250" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2251" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2251">
+        <v>6001056412919</v>
+      </c>
+      <c r="B2251">
+        <v>71093406</v>
+      </c>
+      <c r="C2251" t="s">
+        <v>4495</v>
+      </c>
+      <c r="D2251">
+        <v>4500</v>
+      </c>
+      <c r="E2251" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2252" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2252">
+        <v>6001056412933</v>
+      </c>
+      <c r="B2252">
+        <v>71093407</v>
+      </c>
+      <c r="C2252" t="s">
+        <v>4496</v>
+      </c>
+      <c r="D2252">
+        <v>4500</v>
+      </c>
+      <c r="E2252" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2253" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2253">
+        <v>6001056412926</v>
+      </c>
+      <c r="B2253">
+        <v>71093408</v>
+      </c>
+      <c r="C2253" t="s">
+        <v>4497</v>
+      </c>
+      <c r="D2253">
+        <v>4500</v>
+      </c>
+      <c r="E2253" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2254">
+        <v>6009704171294</v>
+      </c>
+      <c r="B2254">
+        <v>71093409</v>
+      </c>
+      <c r="C2254" t="s">
+        <v>4498</v>
+      </c>
+      <c r="D2254">
+        <v>10500</v>
+      </c>
+      <c r="E2254" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2255" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2255">
+        <v>6001056201001</v>
+      </c>
+      <c r="B2255">
+        <v>71093410</v>
+      </c>
+      <c r="C2255" t="s">
+        <v>4499</v>
+      </c>
+      <c r="D2255">
+        <v>10500</v>
+      </c>
+      <c r="E2255" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2256" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2256">
+        <v>6009704171874</v>
+      </c>
+      <c r="B2256">
+        <v>71093411</v>
+      </c>
+      <c r="C2256" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D2256">
+        <v>4690</v>
+      </c>
+      <c r="E2256" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2257">
+        <v>6009702443447</v>
+      </c>
+      <c r="B2257">
+        <v>71093412</v>
+      </c>
+      <c r="C2257" t="s">
+        <v>4501</v>
+      </c>
+      <c r="D2257">
+        <v>28500</v>
+      </c>
+      <c r="E2257" t="s">
+        <v>4494</v>
+      </c>
+    </row>
+    <row r="2258" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2258">
+        <v>6091303395027</v>
+      </c>
+      <c r="B2258">
+        <v>71093413</v>
+      </c>
+      <c r="C2258" t="s">
+        <v>4502</v>
+      </c>
+      <c r="D2258">
+        <v>4900</v>
+      </c>
+      <c r="E2258" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>